<commit_message>
ci: add GitHub Actions workflow and CI-controlled test execution
</commit_message>
<xml_diff>
--- a/DemoData/TestPlan.xlsx
+++ b/DemoData/TestPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sdet-framework-reference\DemoData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBF9DE5-BABA-4751-8752-D1E0EF13A97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDEF72B0-D8F7-4FFA-9446-A9846AF6D77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5904" yWindow="0" windowWidth="17280" windowHeight="9960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestDir" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>TestName</t>
   </si>
@@ -167,6 +167,18 @@
   </si>
   <si>
     <t>add_item_to_cart</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>默認為index=0加入第一個商品</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Parameter</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>index=0</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -234,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -248,6 +260,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -633,18 +648,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D653F17-7651-4C82-8B74-0BA06AE6A92F}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="36.875" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.875" style="2"/>
-    <col min="5" max="5" width="30.5" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="36.875" style="2"/>
+    <col min="4" max="4" width="22.25" style="2" customWidth="1"/>
+    <col min="5" max="5" width="36.875" style="2"/>
+    <col min="6" max="6" width="30.5" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="36.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -655,13 +671,16 @@
         <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -671,11 +690,12 @@
       <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="D2" s="3"/>
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -685,8 +705,9 @@
       <c r="C3" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
@@ -696,7 +717,13 @@
       <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Case 2-2 Web recording playback automation complete
- Smart language switching to Traditional Chinese

- Smart waiting for View tab, Server, and Camera

- Multi-strategy XPath for stability

- Timeline green block click and pause button

- Browser auto-maximize and bring to front
</commit_message>
<xml_diff>
--- a/DemoData/TestPlan.xlsx
+++ b/DemoData/TestPlan.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\nxwitness-demo\DemoData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54EBDDD8-B81D-4D6E-B7D1-4EECD6624003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09511917-5EBB-47FD-B053-693FA02B639F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4896" yWindow="3720" windowWidth="17280" windowHeight="9960" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1944" yWindow="1884" windowWidth="17280" windowHeight="9960" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestDir" sheetId="1" r:id="rId1"/>
     <sheet name="Case1" sheetId="2" r:id="rId2"/>
-    <sheet name="Case2" sheetId="4" r:id="rId3"/>
-    <sheet name="Case4" sheetId="5" r:id="rId4"/>
-    <sheet name="Translate" sheetId="3" r:id="rId5"/>
+    <sheet name="Case2" sheetId="3" r:id="rId3"/>
+    <sheet name="Case4" sheetId="4" r:id="rId4"/>
+    <sheet name="Translate" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="64">
   <si>
     <t>FunctionalClassification</t>
   </si>
@@ -68,6 +68,36 @@
     <t>回放錄影事件後停止</t>
   </si>
   <si>
+    <t>Case2</t>
+  </si>
+  <si>
+    <t>Test case 2-1</t>
+  </si>
+  <si>
+    <t>進⼊ Nx Cloud</t>
+  </si>
+  <si>
+    <t>Test case 2-2</t>
+  </si>
+  <si>
+    <t>調閱⼀個錄影事件回放</t>
+  </si>
+  <si>
+    <t>Case4</t>
+  </si>
+  <si>
+    <t>Test case 4-1</t>
+  </si>
+  <si>
+    <t>Mobile-Nx Witness mobile 登入 Nx Cloud</t>
+  </si>
+  <si>
+    <t>Test case 4-2</t>
+  </si>
+  <si>
+    <t>調閱一個錄影事件回放 (Mobile Android)</t>
+  </si>
+  <si>
     <t>StepNo</t>
   </si>
   <si>
@@ -107,290 +137,92 @@
     <t>camera_name=usb_cam;playback_duration=7</t>
   </si>
   <si>
+    <t>login_nx_cloud_web</t>
+  </si>
+  <si>
+    <t>review_recording_playback</t>
+  </si>
+  <si>
+    <t>login_mobile</t>
+  </si>
+  <si>
+    <t>select_server_and_camera</t>
+  </si>
+  <si>
+    <t>server_name=LAPTOP-QRJN5735;camera_name=usb_cam</t>
+  </si>
+  <si>
+    <t>playback_with_calendar</t>
+  </si>
+  <si>
+    <t>days_ago=17</t>
+  </si>
+  <si>
+    <t>ActionKey</t>
+  </si>
+  <si>
     <t>ActionMethod</t>
   </si>
   <si>
-    <t>nx_poc</t>
+    <t>login</t>
   </si>
   <si>
     <t>run_ensure_login_step</t>
   </si>
   <si>
+    <t>settings</t>
+  </si>
+  <si>
     <t>run_change_language_step</t>
   </si>
   <si>
+    <t>camera</t>
+  </si>
+  <si>
     <t>run_enable_usb_webcam_step</t>
   </si>
   <si>
+    <t>license</t>
+  </si>
+  <si>
     <t>run_activate_free_license_step</t>
   </si>
   <si>
+    <t>recording</t>
+  </si>
+  <si>
     <t>run_enable_recording_step</t>
   </si>
   <si>
     <t>run_playback_recording_step</t>
   </si>
   <si>
-    <t>自動登入伺服器並切換繁體中文</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>Case</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Test case </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2-1</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>進</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft JhengHei UI"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>⼊</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="新細明體"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Nx Cloud</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <t>cloud</t>
   </si>
   <si>
     <t>run_enter_nx_cloud_step</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>login_nx_cloud_web</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Test case </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2-2</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>調閱</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft JhengHei UI"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>⼀</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft JhengHei UI"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>個錄影事件回放</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>run_review_recording_playback_step</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>review_recording_playback</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>Case</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>4</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Test case </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>4-1</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Test case </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>4-2</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>調閱一個錄影事件回放 (Mobile Android)</t>
   </si>
   <si>
     <t>nx_mobile</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>run_login_step</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ActionKey</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>login_mobile</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>run_select_server_and_camera_step</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>select_server_and_camera</t>
   </si>
   <si>
     <t>run_playback_with_calendar_step</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>playback_with_calendar</t>
-  </si>
-  <si>
-    <t>playback_with_calendar</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>server_name=LAPTOP-QRJN5735</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>;camera_name=usb_cam</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>days_ago=17</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>Mobile</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="新細明體"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Nx Witness mobile 登入 Nx Cloud</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>調閱一個錄影事件回放 (Mobile Android)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,24 +245,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Microsoft YaHei"/>
-      <family val="2"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Microsoft JhengHei UI"/>
-      <family val="2"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Microsoft JhengHei UI"/>
-      <family val="2"/>
+      <name val="新細明體"/>
+      <family val="1"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -442,12 +260,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -474,7 +307,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -849,54 +684,54 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -918,13 +753,13 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -938,10 +773,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -949,16 +784,16 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -972,10 +807,10 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -989,10 +824,10 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1006,10 +841,10 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1023,7 +858,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1037,10 +872,10 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1054,10 +889,10 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -1071,10 +906,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1088,10 +923,10 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1101,7 +936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D1B7B97-A634-4770-83D9-61FF40525F35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1119,41 +954,41 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B2" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1163,7 +998,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B729A69C-2FFD-487C-BA15-BD8AA698CAC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1180,61 +1015,61 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1244,145 +1079,144 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.375" customWidth="1"/>
-    <col min="2" max="2" width="18.625" customWidth="1"/>
-    <col min="3" max="3" width="29.25" customWidth="1"/>
+    <col min="1" max="1" width="26.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" t="s">
-        <v>27</v>
+      <c r="A1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>